<commit_message>
Updated README and test cases SauceLab App
</commit_message>
<xml_diff>
--- a/src/test/resources/test_data/data.xlsx
+++ b/src/test/resources/test_data/data.xlsx
@@ -1,26 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29415"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30215"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ANHTESTER\Appium\AppiumJava122024_Multi_Platform\src\test\resources\test_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A680FEF7-5CB8-41F9-9CA0-5AFD655D20E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BFF41503-4EA5-4D09-9938-E4C06B4F71AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4452" yWindow="2304" windowWidth="22704" windowHeight="13872" firstSheet="3" activeTab="3" xr2:uid="{5D795E49-F5D6-486B-B630-D84533204838}"/>
+    <workbookView xWindow="4452" yWindow="2304" windowWidth="22704" windowHeight="13872" firstSheet="4" activeTab="4" xr2:uid="{5D795E49-F5D6-486B-B630-D84533204838}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
     <sheet name="Table" sheetId="2" r:id="rId2"/>
     <sheet name="Product" sheetId="3" r:id="rId3"/>
     <sheet name="Login_Excel" sheetId="4" r:id="rId4"/>
+    <sheet name="Login_MyDemoApp" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="30">
   <si>
     <t>TEST_CASE</t>
   </si>
@@ -68,6 +69,9 @@
     <t>admin123</t>
   </si>
   <si>
+    <t>Failed</t>
+  </si>
+  <si>
     <t>123456</t>
   </si>
   <si>
@@ -113,14 +117,25 @@
     <t>password2</t>
   </si>
   <si>
-    <t>Failed</t>
+    <t>MESSAGE</t>
+  </si>
+  <si>
+    <t>bod@example.com</t>
+  </si>
+  <si>
+    <t>alice@example.com</t>
+  </si>
+  <si>
+    <t>Sorry this user has been locked out.</t>
+  </si>
+  <si>
+    <t>visual@example.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <sz val="14"/>
@@ -139,7 +154,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -148,9 +163,6 @@
     </fill>
     <fill>
       <patternFill patternType="none"/>
-    </fill>
-    <fill>
-      <patternFill/>
     </fill>
   </fills>
   <borders count="1">
@@ -172,11 +184,9 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -495,11 +505,11 @@
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="17.45"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="30.7265625"/>
-    <col min="2" max="2" customWidth="true" width="14.36328125"/>
-    <col min="3" max="3" customWidth="true" width="15.54296875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="18.6328125"/>
-    <col min="5" max="5" customWidth="true" width="10.26953125"/>
+    <col min="1" max="1" width="30.7265625" customWidth="1"/>
+    <col min="2" max="2" width="14.36328125" customWidth="1"/>
+    <col min="3" max="3" width="15.54296875" customWidth="1"/>
+    <col min="4" max="4" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.26953125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -517,39 +527,39 @@
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s" s="0">
+      <c r="C2" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:4">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s">
         <v>7</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" t="s" s="0">
+      <c r="C3" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="5" t="s">
-        <v>24</v>
+      <c r="D3" s="3" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:4">
-      <c r="B4" t="s" s="0">
+      <c r="B4" t="s">
         <v>5</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -562,32 +572,32 @@
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="17.45"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="15.26953125"/>
-    <col min="2" max="2" customWidth="true" width="11.54296875"/>
+    <col min="1" max="1" width="15.26953125" customWidth="1"/>
+    <col min="2" max="2" width="11.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" t="s" s="0">
-        <v>12</v>
+      <c r="A2" t="s">
+        <v>13</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" t="s" s="0">
-        <v>14</v>
+      <c r="A3" t="s">
+        <v>15</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -601,32 +611,32 @@
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="17.45"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="16.08984375"/>
-    <col min="2" max="2" customWidth="true" width="13.36328125"/>
+    <col min="1" max="1" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.36328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" t="s" s="0">
-        <v>18</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -639,8 +649,8 @@
   <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="17.45"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="14.36328125"/>
-    <col min="2" max="2" customWidth="true" width="15.54296875"/>
+    <col min="1" max="1" width="14.36328125" customWidth="1"/>
+    <col min="2" max="2" width="15.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -652,46 +662,105 @@
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" t="s" s="0">
-        <v>19</v>
+      <c r="A4" t="s">
+        <v>20</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="B5" t="s" s="0">
+      <c r="A5" t="s">
         <v>21</v>
       </c>
+      <c r="B5" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" t="s" s="0">
-        <v>22</v>
-      </c>
-      <c r="B6" t="s" s="0">
+      <c r="A6" t="s">
         <v>23</v>
+      </c>
+      <c r="B6" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{616F1FF8-0DE8-424B-BEC1-DF914F7409E4}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="18"/>
+  <cols>
+    <col min="1" max="1" width="17.1796875" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="28.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2">
+        <v>10203040</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="21" customHeight="1">
+      <c r="A3" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3">
+        <v>10203040</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4">
+        <v>10203040</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{d9378963-1951-4715-a8fd-de017d62dd42}" enabled="1" method="Privileged" siteId="{f4308c54-0208-43d3-afad-1f8df2f678b7}" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>